<commit_message>
Add explicit Coresignal firmographic reports
</commit_message>
<xml_diff>
--- a/Firmographic/reports/full_10_company_report/hpi_10_company_firmographic_api_report_revised.xlsx
+++ b/Firmographic/reports/full_10_company_report/hpi_10_company_firmographic_api_report_revised.xlsx
@@ -34024,12 +34024,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr"/>
@@ -34127,12 +34127,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr"/>
@@ -34230,12 +34230,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
@@ -34333,12 +34333,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr"/>
@@ -34436,12 +34436,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
@@ -34539,12 +34539,12 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
@@ -34642,12 +34642,12 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr"/>
@@ -34745,12 +34745,12 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr"/>
@@ -34848,12 +34848,12 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr"/>
@@ -34951,12 +34951,12 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T07:48:23Z</t>
+          <t>2026-06-13T08:00:55Z</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr"/>

</xml_diff>